<commit_message>
location and person preference indicators, fix location specs
</commit_message>
<xml_diff>
--- a/public/seating-template.xlsx
+++ b/public/seating-template.xlsx
@@ -664,7 +664,7 @@
         <v>Location Needs</v>
       </c>
       <c r="B9" t="str">
-        <v>HARD RULE. Allowed tables. Table numbers (e.g. "1, 2, 3") or keywords. Multiple lines in one cell must ALL be satisfied.</v>
+        <v>HARD RULE. Allowed tables. Table numbers and/or keywords, comma-separated (e.g. "1, 2, 3" or "front, middle"); anything on the same line counts. Multiple lines in one cell must ALL be satisfied ("front" and "middle" on separate lines allows no table).</v>
       </c>
     </row>
     <row r="10">
@@ -672,7 +672,7 @@
         <v>Location Preference</v>
       </c>
       <c r="B10" t="str">
-        <v>Soft preference, used for highlighting only. Same values as Location Needs; multiple lines = any of them.</v>
+        <v>Soft preference: shown under the student's name as "L: 1, 2, 3" (green when met, red when not; tables ruled out by Location Needs are dropped), and preferred tables are tinted light green while dragging the student; not enforced by Randomize. Same values as Location Needs; everything listed counts, whether on the same line or separate lines.</v>
       </c>
     </row>
     <row r="11">
@@ -680,7 +680,7 @@
         <v>Person Preference</v>
       </c>
       <c r="B11" t="str">
-        <v>Stored but not currently used by the seating logic.</v>
+        <v>Soft preference: names the student would like to sit with, separated by commas or new lines, written "First Last". Shown under the student's name as "P: 1/3" (people at the same table / people listed; green if at least one, red if none) and highlighted green while dragging the student; not enforced by Randomize.</v>
       </c>
     </row>
     <row r="12">

</xml_diff>